<commit_message>
Added building A CAD room glare values to excel
</commit_message>
<xml_diff>
--- a/Excel/Building_A_B_Carpark_Existing_Lighting.xlsx
+++ b/Excel/Building_A_B_Carpark_Existing_Lighting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23E3571-EFBD-4E3D-B9E5-7C3E2498E5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC5106B-583F-4D17-A2EA-8855C04F5852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -646,7 +643,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -847,7 +844,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -949,19 +946,13 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="9" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -973,7 +964,16 @@
     <xf numFmtId="2" fontId="3" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -985,35 +985,7 @@
     <cellStyle name="Normal 5" xfId="4" xr:uid="{ED6D2035-F9DA-4B1D-B2ED-B5DB87628F59}"/>
     <cellStyle name="Normal 6" xfId="5" xr:uid="{FCC80704-4661-421C-AAE8-B6CB6410940C}"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -1224,7 +1196,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB36"/>
-  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -1237,40 +1209,40 @@
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="8.3125" customWidth="1"/>
+    <col min="17" max="17" width="8.296875" customWidth="1"/>
     <col min="18" max="20" width="12" customWidth="1"/>
     <col min="21" max="22" width="14" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="20.65">
-      <c r="A1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-    </row>
-    <row r="2" spans="1:28" ht="41.65">
+    <row r="1" spans="1:28" ht="21">
+      <c r="A1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+    </row>
+    <row r="2" spans="1:28" ht="41.4">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1356,7 +1328,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="27">
+    <row r="3" spans="1:28" ht="27.6">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -1425,14 +1397,14 @@
         <v/>
       </c>
       <c r="AA3" s="20" t="str">
-        <f>IF(OR(S3="",Z3=""),"",S3-Z3)</f>
+        <f t="shared" ref="AA3:AA36" si="1">IF(OR(S3="",Z3=""),"",S3-Z3)</f>
         <v/>
       </c>
       <c r="AB3" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="27">
+    <row r="4" spans="1:28" ht="27.6">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -1508,14 +1480,14 @@
         <v/>
       </c>
       <c r="AA4" s="20" t="str">
-        <f>IF(OR(S4="",Z4=""),"",S4-Z4)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB4" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.5">
+    <row r="5" spans="1:28" ht="26.4">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -1566,7 +1538,7 @@
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="20">
-        <f t="shared" ref="S5:S35" si="1">IF(OR(N5="",O5=""),"",N5*O5)</f>
+        <f t="shared" ref="S5:S35" si="2">IF(OR(N5="",O5=""),"",N5*O5)</f>
         <v>72</v>
       </c>
       <c r="T5" s="27">
@@ -1580,18 +1552,18 @@
       <c r="X5" s="9"/>
       <c r="Y5" s="20"/>
       <c r="Z5" s="20" t="str">
-        <f t="shared" ref="Z5:Z36" si="2">IF(OR(X5="",Y5=""),"",X5*Y5)</f>
+        <f t="shared" ref="Z5:Z36" si="3">IF(OR(X5="",Y5=""),"",X5*Y5)</f>
         <v/>
       </c>
       <c r="AA5" s="20" t="str">
-        <f>IF(OR(S5="",Z5=""),"",S5-Z5)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB5" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.5">
+    <row r="6" spans="1:28" ht="26.4">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -1642,7 +1614,7 @@
       <c r="Q6" s="24"/>
       <c r="R6" s="24"/>
       <c r="S6" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T6" s="27">
@@ -1656,18 +1628,18 @@
       <c r="X6" s="9"/>
       <c r="Y6" s="20"/>
       <c r="Z6" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA6" s="20" t="str">
-        <f>IF(OR(S6="",Z6=""),"",S6-Z6)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB6" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.5">
+    <row r="7" spans="1:28" ht="26.4">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -1718,7 +1690,7 @@
       <c r="Q7" s="24"/>
       <c r="R7" s="24"/>
       <c r="S7" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T7" s="27">
@@ -1732,18 +1704,18 @@
       <c r="X7" s="9"/>
       <c r="Y7" s="20"/>
       <c r="Z7" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA7" s="20" t="str">
-        <f>IF(OR(S7="",Z7=""),"",S7-Z7)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB7" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.5">
+    <row r="8" spans="1:28" ht="26.4">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -1794,7 +1766,7 @@
       <c r="Q8" s="24"/>
       <c r="R8" s="24"/>
       <c r="S8" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T8" s="27">
@@ -1808,18 +1780,18 @@
       <c r="X8" s="9"/>
       <c r="Y8" s="20"/>
       <c r="Z8" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA8" s="20" t="str">
-        <f>IF(OR(S8="",Z8=""),"",S8-Z8)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB8" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.5">
+    <row r="9" spans="1:28" ht="26.4">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -1870,7 +1842,7 @@
       <c r="Q9" s="24"/>
       <c r="R9" s="24"/>
       <c r="S9" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T9" s="27">
@@ -1884,18 +1856,18 @@
       <c r="X9" s="9"/>
       <c r="Y9" s="20"/>
       <c r="Z9" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA9" s="20" t="str">
-        <f>IF(OR(S9="",Z9=""),"",S9-Z9)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB9" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="27">
+    <row r="10" spans="1:28" ht="27.6">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1967,18 +1939,18 @@
       <c r="X10" s="9"/>
       <c r="Y10" s="20"/>
       <c r="Z10" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA10" s="20" t="str">
-        <f>IF(OR(S10="",Z10=""),"",S10-Z10)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB10" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.5">
+    <row r="11" spans="1:28" ht="26.4">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -2029,7 +2001,7 @@
       <c r="Q11" s="24"/>
       <c r="R11" s="24"/>
       <c r="S11" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T11" s="27">
@@ -2046,14 +2018,14 @@
         <v/>
       </c>
       <c r="AA11" s="20" t="str">
-        <f>IF(OR(S11="",Z11=""),"",S11-Z11)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB11" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.5">
+    <row r="12" spans="1:28" ht="26.4">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -2104,7 +2076,7 @@
       <c r="Q12" s="24"/>
       <c r="R12" s="24"/>
       <c r="S12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T12" s="27">
@@ -2122,14 +2094,14 @@
         <v>#REF!</v>
       </c>
       <c r="AA12" s="20" t="e">
-        <f>IF(OR(S12="",Z12=""),"",S12-Z12)</f>
+        <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
       <c r="AB12" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.5">
+    <row r="13" spans="1:28" ht="26.4">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -2180,32 +2152,34 @@
       <c r="Q13" s="24"/>
       <c r="R13" s="24"/>
       <c r="S13" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T13" s="27">
         <v>743</v>
       </c>
       <c r="U13" s="27"/>
-      <c r="V13" s="27"/>
+      <c r="V13" s="44">
+        <v>19.399999999999999</v>
+      </c>
       <c r="W13" s="9" t="s">
         <v>56</v>
       </c>
       <c r="X13" s="9"/>
       <c r="Y13" s="20"/>
       <c r="Z13" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA13" s="20" t="str">
-        <f>IF(OR(S13="",Z13=""),"",S13-Z13)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB13" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.5">
+    <row r="14" spans="1:28" ht="26.4">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -2256,32 +2230,34 @@
       <c r="Q14" s="24"/>
       <c r="R14" s="24"/>
       <c r="S14" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>864</v>
       </c>
       <c r="T14" s="27">
         <v>1088</v>
       </c>
       <c r="U14" s="27"/>
-      <c r="V14" s="27"/>
+      <c r="V14" s="44">
+        <v>19.5</v>
+      </c>
       <c r="W14" s="9" t="s">
         <v>56</v>
       </c>
       <c r="X14" s="9"/>
       <c r="Y14" s="20"/>
       <c r="Z14" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA14" s="20" t="str">
-        <f>IF(OR(S14="",Z14=""),"",S14-Z14)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB14" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.5">
+    <row r="15" spans="1:28" ht="26.4">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -2332,7 +2308,7 @@
       <c r="Q15" s="24"/>
       <c r="R15" s="24"/>
       <c r="S15" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="T15" s="27">
@@ -2346,18 +2322,18 @@
       <c r="X15" s="9"/>
       <c r="Y15" s="20"/>
       <c r="Z15" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA15" s="20" t="str">
-        <f>IF(OR(S15="",Z15=""),"",S15-Z15)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB15" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.5">
+    <row r="16" spans="1:28" ht="26.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2408,7 +2384,7 @@
       <c r="Q16" s="24"/>
       <c r="R16" s="24"/>
       <c r="S16" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="T16" s="27">
@@ -2422,18 +2398,18 @@
       <c r="X16" s="9"/>
       <c r="Y16" s="20"/>
       <c r="Z16" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA16" s="20" t="str">
-        <f>IF(OR(S16="",Z16=""),"",S16-Z16)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB16" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="27">
+    <row r="17" spans="1:28" ht="27.6">
       <c r="A17" s="6" t="s">
         <v>78</v>
       </c>
@@ -2484,7 +2460,7 @@
       <c r="Q17" s="24"/>
       <c r="R17" s="24"/>
       <c r="S17" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T17" s="27">
@@ -2498,18 +2474,18 @@
       <c r="X17" s="9"/>
       <c r="Y17" s="20"/>
       <c r="Z17" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA17" s="20" t="str">
-        <f>IF(OR(S17="",Z17=""),"",S17-Z17)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB17" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="27">
+    <row r="18" spans="1:28" ht="27.6">
       <c r="A18" s="6" t="s">
         <v>78</v>
       </c>
@@ -2560,7 +2536,7 @@
       <c r="Q18" s="24"/>
       <c r="R18" s="24"/>
       <c r="S18" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T18" s="27">
@@ -2574,18 +2550,18 @@
       <c r="X18" s="9"/>
       <c r="Y18" s="20"/>
       <c r="Z18" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA18" s="20" t="str">
-        <f>IF(OR(S18="",Z18=""),"",S18-Z18)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB18" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.5">
+    <row r="19" spans="1:28" ht="26.4">
       <c r="A19" s="6" t="s">
         <v>78</v>
       </c>
@@ -2636,7 +2612,7 @@
       <c r="Q19" s="24"/>
       <c r="R19" s="24"/>
       <c r="S19" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T19" s="27">
@@ -2650,18 +2626,18 @@
       <c r="X19" s="9"/>
       <c r="Y19" s="20"/>
       <c r="Z19" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA19" s="20" t="str">
-        <f>IF(OR(S19="",Z19=""),"",S19-Z19)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB19" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.5">
+    <row r="20" spans="1:28" ht="26.4">
       <c r="A20" s="6" t="s">
         <v>78</v>
       </c>
@@ -2712,7 +2688,7 @@
       <c r="Q20" s="24"/>
       <c r="R20" s="24"/>
       <c r="S20" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1008</v>
       </c>
       <c r="T20" s="27">
@@ -2726,18 +2702,18 @@
       <c r="X20" s="9"/>
       <c r="Y20" s="20"/>
       <c r="Z20" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA20" s="20" t="str">
-        <f>IF(OR(S20="",Z20=""),"",S20-Z20)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB20" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="27">
+    <row r="21" spans="1:28" ht="27.6">
       <c r="A21" s="6" t="s">
         <v>78</v>
       </c>
@@ -2788,7 +2764,7 @@
       <c r="Q21" s="24"/>
       <c r="R21" s="24"/>
       <c r="S21" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T21" s="27">
@@ -2802,18 +2778,18 @@
       <c r="X21" s="9"/>
       <c r="Y21" s="20"/>
       <c r="Z21" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA21" s="20" t="str">
-        <f>IF(OR(S21="",Z21=""),"",S21-Z21)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB21" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.5">
+    <row r="22" spans="1:28" ht="26.4">
       <c r="A22" s="6" t="s">
         <v>78</v>
       </c>
@@ -2864,7 +2840,7 @@
       <c r="Q22" s="24"/>
       <c r="R22" s="24"/>
       <c r="S22" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>144</v>
       </c>
       <c r="T22" s="27">
@@ -2878,18 +2854,18 @@
       <c r="X22" s="9"/>
       <c r="Y22" s="20"/>
       <c r="Z22" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA22" s="20" t="str">
-        <f>IF(OR(S22="",Z22=""),"",S22-Z22)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB22" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.5">
+    <row r="23" spans="1:28" ht="26.4">
       <c r="A23" s="6" t="s">
         <v>78</v>
       </c>
@@ -2940,7 +2916,7 @@
       <c r="Q23" s="24"/>
       <c r="R23" s="24"/>
       <c r="S23" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>864</v>
       </c>
       <c r="T23" s="27">
@@ -2954,18 +2930,18 @@
       <c r="X23" s="9"/>
       <c r="Y23" s="20"/>
       <c r="Z23" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA23" s="20" t="str">
-        <f>IF(OR(S23="",Z23=""),"",S23-Z23)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB23" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.5">
+    <row r="24" spans="1:28" ht="26.4">
       <c r="A24" s="6" t="s">
         <v>78</v>
       </c>
@@ -3016,7 +2992,7 @@
       <c r="Q24" s="24"/>
       <c r="R24" s="24"/>
       <c r="S24" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T24" s="27">
@@ -3030,18 +3006,18 @@
       <c r="X24" s="9"/>
       <c r="Y24" s="20"/>
       <c r="Z24" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA24" s="20" t="str">
-        <f>IF(OR(S24="",Z24=""),"",S24-Z24)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB24" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.5">
+    <row r="25" spans="1:28" ht="26.4">
       <c r="A25" s="6" t="s">
         <v>78</v>
       </c>
@@ -3092,7 +3068,7 @@
       <c r="Q25" s="24"/>
       <c r="R25" s="24"/>
       <c r="S25" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T25" s="27">
@@ -3106,18 +3082,18 @@
       <c r="X25" s="9"/>
       <c r="Y25" s="20"/>
       <c r="Z25" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA25" s="20" t="str">
-        <f>IF(OR(S25="",Z25=""),"",S25-Z25)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB25" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.5">
+    <row r="26" spans="1:28" ht="26.4">
       <c r="A26" s="6" t="s">
         <v>78</v>
       </c>
@@ -3168,32 +3144,34 @@
       <c r="Q26" s="24"/>
       <c r="R26" s="24"/>
       <c r="S26" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1152</v>
       </c>
       <c r="T26" s="27">
         <v>455</v>
       </c>
       <c r="U26" s="27"/>
-      <c r="V26" s="27"/>
+      <c r="V26" s="44">
+        <v>22</v>
+      </c>
       <c r="W26" s="9" t="s">
         <v>56</v>
       </c>
       <c r="X26" s="9"/>
       <c r="Y26" s="20"/>
       <c r="Z26" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA26" s="20" t="str">
-        <f>IF(OR(S26="",Z26=""),"",S26-Z26)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB26" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="27">
+    <row r="27" spans="1:28" ht="27.6">
       <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
@@ -3244,7 +3222,7 @@
       <c r="Q27" s="24"/>
       <c r="R27" s="24"/>
       <c r="S27" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T27" s="27">
@@ -3258,18 +3236,18 @@
       <c r="X27" s="9"/>
       <c r="Y27" s="20"/>
       <c r="Z27" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA27" s="20" t="str">
-        <f>IF(OR(S27="",Z27=""),"",S27-Z27)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB27" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.5">
+    <row r="28" spans="1:28" ht="26.4">
       <c r="A28" s="6" t="s">
         <v>78</v>
       </c>
@@ -3320,7 +3298,7 @@
       <c r="Q28" s="24"/>
       <c r="R28" s="24"/>
       <c r="S28" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1152</v>
       </c>
       <c r="T28" s="27">
@@ -3334,18 +3312,18 @@
       <c r="X28" s="9"/>
       <c r="Y28" s="20"/>
       <c r="Z28" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA28" s="20" t="str">
-        <f>IF(OR(S28="",Z28=""),"",S28-Z28)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="27">
+    <row r="29" spans="1:28" ht="27.6">
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
@@ -3396,7 +3374,7 @@
       <c r="Q29" s="24"/>
       <c r="R29" s="24"/>
       <c r="S29" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T29" s="27">
@@ -3410,18 +3388,18 @@
       <c r="X29" s="9"/>
       <c r="Y29" s="20"/>
       <c r="Z29" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA29" s="20" t="str">
-        <f>IF(OR(S29="",Z29=""),"",S29-Z29)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB29" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="25.5">
+    <row r="30" spans="1:28" ht="26.4">
       <c r="A30" s="6" t="s">
         <v>78</v>
       </c>
@@ -3472,7 +3450,7 @@
       <c r="Q30" s="24"/>
       <c r="R30" s="24"/>
       <c r="S30" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T30" s="27">
@@ -3486,18 +3464,18 @@
       <c r="X30" s="9"/>
       <c r="Y30" s="20"/>
       <c r="Z30" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA30" s="20" t="str">
-        <f>IF(OR(S30="",Z30=""),"",S30-Z30)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB30" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="25.5">
+    <row r="31" spans="1:28" ht="26.4">
       <c r="A31" s="6" t="s">
         <v>78</v>
       </c>
@@ -3548,7 +3526,7 @@
       <c r="Q31" s="24"/>
       <c r="R31" s="24"/>
       <c r="S31" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T31" s="27">
@@ -3562,18 +3540,18 @@
       <c r="X31" s="9"/>
       <c r="Y31" s="20"/>
       <c r="Z31" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA31" s="20" t="str">
-        <f>IF(OR(S31="",Z31=""),"",S31-Z31)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB31" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="25.5">
+    <row r="32" spans="1:28" ht="26.4">
       <c r="A32" s="6" t="s">
         <v>78</v>
       </c>
@@ -3624,7 +3602,7 @@
       <c r="Q32" s="24"/>
       <c r="R32" s="24"/>
       <c r="S32" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T32" s="27">
@@ -3638,18 +3616,18 @@
       <c r="X32" s="9"/>
       <c r="Y32" s="20"/>
       <c r="Z32" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA32" s="20" t="str">
-        <f>IF(OR(S32="",Z32=""),"",S32-Z32)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB32" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="25.5">
+    <row r="33" spans="1:28" ht="26.4">
       <c r="A33" s="6" t="s">
         <v>78</v>
       </c>
@@ -3700,7 +3678,7 @@
       <c r="Q33" s="24"/>
       <c r="R33" s="24"/>
       <c r="S33" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T33" s="27">
@@ -3714,18 +3692,18 @@
       <c r="X33" s="9"/>
       <c r="Y33" s="20"/>
       <c r="Z33" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA33" s="20" t="str">
-        <f>IF(OR(S33="",Z33=""),"",S33-Z33)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB33" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="25.5">
+    <row r="34" spans="1:28" ht="26.4">
       <c r="A34" s="6" t="s">
         <v>78</v>
       </c>
@@ -3776,7 +3754,7 @@
       <c r="Q34" s="24"/>
       <c r="R34" s="24"/>
       <c r="S34" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T34" s="27">
@@ -3790,18 +3768,18 @@
       <c r="X34" s="9"/>
       <c r="Y34" s="20"/>
       <c r="Z34" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA34" s="20" t="str">
-        <f>IF(OR(S34="",Z34=""),"",S34-Z34)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB34" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="25.5">
+    <row r="35" spans="1:28" ht="26.4">
       <c r="A35" s="6" t="s">
         <v>78</v>
       </c>
@@ -3852,7 +3830,7 @@
       <c r="Q35" s="24"/>
       <c r="R35" s="24"/>
       <c r="S35" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="T35" s="27">
@@ -3866,18 +3844,18 @@
       <c r="X35" s="9"/>
       <c r="Y35" s="20"/>
       <c r="Z35" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA35" s="20" t="str">
-        <f>IF(OR(S35="",Z35=""),"",S35-Z35)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB35" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="25.5">
+    <row r="36" spans="1:28" ht="26.4">
       <c r="A36" s="11" t="s">
         <v>78</v>
       </c>
@@ -3942,11 +3920,11 @@
       <c r="X36" s="14"/>
       <c r="Y36" s="21"/>
       <c r="Z36" s="21" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA36" s="21" t="str">
-        <f>IF(OR(S36="",Z36=""),"",S36-Z36)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB36" s="15" t="s">
@@ -3958,10 +3936,10 @@
     <mergeCell ref="A1:W1"/>
   </mergeCells>
   <conditionalFormatting sqref="T4:V36">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$T4&lt;$F4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3973,7 +3951,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AB41"/>
-  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -3986,7 +3964,7 @@
     <col min="13" max="13" width="22" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="12" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="14" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="15.6875" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="15.69921875" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="12" hidden="1" customWidth="1"/>
     <col min="19" max="20" width="14" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="24" customWidth="1"/>
@@ -3995,37 +3973,37 @@
     <col min="26" max="26" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="20.65">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:28" ht="21">
+      <c r="A1" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="35"/>
-      <c r="Y1" s="35"/>
-      <c r="Z1" s="35"/>
-    </row>
-    <row r="2" spans="1:28" ht="41.65">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="42"/>
+    </row>
+    <row r="2" spans="1:28" ht="41.4">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -4111,7 +4089,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.5">
+    <row r="3" spans="1:28" ht="26.4">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -4188,14 +4166,14 @@
         <v/>
       </c>
       <c r="AA3" s="20" t="str">
-        <f>IF(OR(S3="",Z3=""),"",S3-Z3)</f>
+        <f t="shared" ref="AA3:AA38" si="2">IF(OR(S3="",Z3=""),"",S3-Z3)</f>
         <v/>
       </c>
       <c r="AB3" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.5">
+    <row r="4" spans="1:28" ht="26.4">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -4240,7 +4218,7 @@
         <v>2</v>
       </c>
       <c r="O4" s="20">
-        <f t="shared" ref="O4:O23" si="2">2*36*N4</f>
+        <f t="shared" ref="O4:O23" si="3">2*36*N4</f>
         <v>144</v>
       </c>
       <c r="P4" s="25" t="s">
@@ -4250,11 +4228,11 @@
         <v>5</v>
       </c>
       <c r="R4" s="24">
-        <f t="shared" ref="R4:R24" si="3">4*36*Q4</f>
+        <f t="shared" ref="R4:R24" si="4">4*36*Q4</f>
         <v>720</v>
       </c>
       <c r="S4" s="20">
-        <f t="shared" ref="S4:S23" si="4">O4+R4</f>
+        <f t="shared" ref="S4:S23" si="5">O4+R4</f>
         <v>864</v>
       </c>
       <c r="T4" s="27">
@@ -4272,14 +4250,14 @@
         <v/>
       </c>
       <c r="AA4" s="20" t="str">
-        <f>IF(OR(S4="",Z4=""),"",S4-Z4)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB4" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.5">
+    <row r="5" spans="1:28" ht="26.4">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -4324,7 +4302,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P5" s="25" t="s">
@@ -4334,11 +4312,11 @@
         <v>1</v>
       </c>
       <c r="R5" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>144</v>
       </c>
       <c r="S5" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>144</v>
       </c>
       <c r="T5" s="27">
@@ -4356,14 +4334,14 @@
         <v/>
       </c>
       <c r="AA5" s="20" t="str">
-        <f>IF(OR(S5="",Z5=""),"",S5-Z5)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB5" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.5">
+    <row r="6" spans="1:28" ht="26.4">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -4408,7 +4386,7 @@
         <v>1</v>
       </c>
       <c r="O6" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P6" s="25" t="s">
@@ -4418,11 +4396,11 @@
         <v>0</v>
       </c>
       <c r="R6" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S6" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T6" s="27">
@@ -4440,14 +4418,14 @@
         <v/>
       </c>
       <c r="AA6" s="20" t="str">
-        <f>IF(OR(S6="",Z6=""),"",S6-Z6)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB6" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.5">
+    <row r="7" spans="1:28" ht="26.4">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -4492,7 +4470,7 @@
         <v>1</v>
       </c>
       <c r="O7" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P7" s="25" t="s">
@@ -4502,11 +4480,11 @@
         <v>0</v>
       </c>
       <c r="R7" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S7" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T7" s="27">
@@ -4524,14 +4502,14 @@
         <v/>
       </c>
       <c r="AA7" s="20" t="str">
-        <f>IF(OR(S7="",Z7=""),"",S7-Z7)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB7" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.5">
+    <row r="8" spans="1:28" ht="26.4">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -4576,7 +4554,7 @@
         <v>1</v>
       </c>
       <c r="O8" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P8" s="25" t="s">
@@ -4586,11 +4564,11 @@
         <v>0</v>
       </c>
       <c r="R8" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S8" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T8" s="27">
@@ -4608,14 +4586,14 @@
         <v/>
       </c>
       <c r="AA8" s="20" t="str">
-        <f>IF(OR(S8="",Z8=""),"",S8-Z8)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB8" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.5">
+    <row r="9" spans="1:28" ht="26.4">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -4660,7 +4638,7 @@
         <v>1</v>
       </c>
       <c r="O9" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P9" s="25" t="s">
@@ -4670,11 +4648,11 @@
         <v>0</v>
       </c>
       <c r="R9" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S9" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T9" s="27">
@@ -4692,14 +4670,14 @@
         <v/>
       </c>
       <c r="AA9" s="20" t="str">
-        <f>IF(OR(S9="",Z9=""),"",S9-Z9)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB9" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.5">
+    <row r="10" spans="1:28" ht="26.4">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -4744,7 +4722,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P10" s="25" t="s">
@@ -4754,11 +4732,11 @@
         <v>4</v>
       </c>
       <c r="R10" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>576</v>
       </c>
       <c r="S10" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>576</v>
       </c>
       <c r="T10" s="27">
@@ -4776,14 +4754,14 @@
         <v/>
       </c>
       <c r="AA10" s="20" t="str">
-        <f>IF(OR(S10="",Z10=""),"",S10-Z10)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB10" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.5">
+    <row r="11" spans="1:28" ht="26.4">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -4803,7 +4781,7 @@
         <v>320</v>
       </c>
       <c r="G11" s="18">
-        <f t="shared" ref="G11" si="5">ROUND(F11/0.8,0)</f>
+        <f t="shared" ref="G11" si="6">ROUND(F11/0.8,0)</f>
         <v>400</v>
       </c>
       <c r="H11" s="8" t="s">
@@ -4828,7 +4806,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P11" s="25" t="s">
@@ -4838,7 +4816,7 @@
         <v>2</v>
       </c>
       <c r="R11" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>288</v>
       </c>
       <c r="S11" s="20">
@@ -4856,18 +4834,18 @@
       <c r="X11" s="9"/>
       <c r="Y11" s="20"/>
       <c r="Z11" s="20" t="str">
-        <f t="shared" ref="Z11" si="6">IF(OR(X11="",Y11=""),"",X11*Y11)</f>
+        <f t="shared" ref="Z11" si="7">IF(OR(X11="",Y11=""),"",X11*Y11)</f>
         <v/>
       </c>
       <c r="AA11" s="20" t="str">
-        <f>IF(OR(S11="",Z11=""),"",S11-Z11)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB11" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.5">
+    <row r="12" spans="1:28" ht="26.4">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -4912,7 +4890,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P12" s="25" t="s">
@@ -4922,11 +4900,11 @@
         <v>6</v>
       </c>
       <c r="R12" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>864</v>
       </c>
       <c r="S12" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>864</v>
       </c>
       <c r="T12" s="27">
@@ -4944,14 +4922,14 @@
         <v/>
       </c>
       <c r="AA12" s="20" t="str">
-        <f>IF(OR(S12="",Z12=""),"",S12-Z12)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB12" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.5">
+    <row r="13" spans="1:28" ht="26.4">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -4996,7 +4974,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P13" s="25" t="s">
@@ -5006,11 +4984,11 @@
         <v>2</v>
       </c>
       <c r="R13" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>288</v>
       </c>
       <c r="S13" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>288</v>
       </c>
       <c r="T13" s="27">
@@ -5028,14 +5006,14 @@
         <v/>
       </c>
       <c r="AA13" s="20" t="str">
-        <f>IF(OR(S13="",Z13=""),"",S13-Z13)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB13" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.5">
+    <row r="14" spans="1:28" ht="26.4">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -5080,7 +5058,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P14" s="25" t="s">
@@ -5090,11 +5068,11 @@
         <v>3</v>
       </c>
       <c r="R14" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>432</v>
       </c>
       <c r="S14" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>432</v>
       </c>
       <c r="T14" s="27">
@@ -5112,14 +5090,14 @@
         <v/>
       </c>
       <c r="AA14" s="20" t="str">
-        <f>IF(OR(S14="",Z14=""),"",S14-Z14)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB14" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.5">
+    <row r="15" spans="1:28" ht="26.4">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -5164,7 +5142,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P15" s="25" t="s">
@@ -5174,11 +5152,11 @@
         <v>2</v>
       </c>
       <c r="R15" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>288</v>
       </c>
       <c r="S15" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>288</v>
       </c>
       <c r="T15" s="27">
@@ -5196,14 +5174,14 @@
         <v/>
       </c>
       <c r="AA15" s="20" t="str">
-        <f>IF(OR(S15="",Z15=""),"",S15-Z15)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB15" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.5">
+    <row r="16" spans="1:28" ht="26.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -5248,7 +5226,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P16" s="25" t="s">
@@ -5258,11 +5236,11 @@
         <v>1</v>
       </c>
       <c r="R16" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>144</v>
       </c>
       <c r="S16" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>144</v>
       </c>
       <c r="T16" s="27">
@@ -5280,14 +5258,14 @@
         <v/>
       </c>
       <c r="AA16" s="20" t="str">
-        <f>IF(OR(S16="",Z16=""),"",S16-Z16)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB16" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.5">
+    <row r="17" spans="1:28" ht="26.4">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -5332,7 +5310,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P17" s="25" t="s">
@@ -5342,11 +5320,11 @@
         <v>4</v>
       </c>
       <c r="R17" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>576</v>
       </c>
       <c r="S17" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>576</v>
       </c>
       <c r="T17" s="27">
@@ -5364,14 +5342,14 @@
         <v/>
       </c>
       <c r="AA17" s="20" t="str">
-        <f>IF(OR(S17="",Z17=""),"",S17-Z17)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB17" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.5">
+    <row r="18" spans="1:28" ht="26.4">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -5416,7 +5394,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P18" s="25" t="s">
@@ -5426,11 +5404,11 @@
         <v>2</v>
       </c>
       <c r="R18" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>288</v>
       </c>
       <c r="S18" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>288</v>
       </c>
       <c r="T18" s="27">
@@ -5448,14 +5426,14 @@
         <v/>
       </c>
       <c r="AA18" s="20" t="str">
-        <f>IF(OR(S18="",Z18=""),"",S18-Z18)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB18" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.5">
+    <row r="19" spans="1:28" ht="26.4">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -5500,7 +5478,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P19" s="25" t="s">
@@ -5510,11 +5488,11 @@
         <v>6</v>
       </c>
       <c r="R19" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>864</v>
       </c>
       <c r="S19" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>864</v>
       </c>
       <c r="T19" s="27">
@@ -5532,14 +5510,14 @@
         <v/>
       </c>
       <c r="AA19" s="20" t="str">
-        <f>IF(OR(S19="",Z19=""),"",S19-Z19)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB19" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.5">
+    <row r="20" spans="1:28" ht="26.4">
       <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
@@ -5584,7 +5562,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P20" s="25" t="s">
@@ -5594,11 +5572,11 @@
         <v>4</v>
       </c>
       <c r="R20" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>576</v>
       </c>
       <c r="S20" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>576</v>
       </c>
       <c r="T20" s="27">
@@ -5616,14 +5594,14 @@
         <v/>
       </c>
       <c r="AA20" s="20" t="str">
-        <f>IF(OR(S20="",Z20=""),"",S20-Z20)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB20" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.5">
+    <row r="21" spans="1:28" ht="26.4">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
@@ -5668,7 +5646,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P21" s="25" t="s">
@@ -5678,11 +5656,11 @@
         <v>1</v>
       </c>
       <c r="R21" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>144</v>
       </c>
       <c r="S21" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>144</v>
       </c>
       <c r="T21" s="27">
@@ -5700,14 +5678,14 @@
         <v/>
       </c>
       <c r="AA21" s="20" t="str">
-        <f>IF(OR(S21="",Z21=""),"",S21-Z21)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB21" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.5">
+    <row r="22" spans="1:28" ht="26.4">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -5752,7 +5730,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P22" s="25" t="s">
@@ -5762,11 +5740,11 @@
         <v>4</v>
       </c>
       <c r="R22" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>576</v>
       </c>
       <c r="S22" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>576</v>
       </c>
       <c r="T22" s="27">
@@ -5784,14 +5762,14 @@
         <v/>
       </c>
       <c r="AA22" s="20" t="str">
-        <f>IF(OR(S22="",Z22=""),"",S22-Z22)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB22" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.5">
+    <row r="23" spans="1:28" ht="26.4">
       <c r="A23" s="6" t="s">
         <v>22</v>
       </c>
@@ -5836,7 +5814,7 @@
         <v>0</v>
       </c>
       <c r="O23" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P23" s="25" t="s">
@@ -5846,11 +5824,11 @@
         <v>2</v>
       </c>
       <c r="R23" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>288</v>
       </c>
       <c r="S23" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>288</v>
       </c>
       <c r="T23" s="27">
@@ -5868,14 +5846,14 @@
         <v/>
       </c>
       <c r="AA23" s="20" t="str">
-        <f>IF(OR(S23="",Z23=""),"",S23-Z23)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB23" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.5">
+    <row r="24" spans="1:28" ht="26.4">
       <c r="A24" s="6" t="s">
         <v>78</v>
       </c>
@@ -5930,7 +5908,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S24" s="20">
@@ -5940,10 +5918,10 @@
       <c r="T24" s="29">
         <v>229</v>
       </c>
-      <c r="U24" s="38">
+      <c r="U24" s="36">
         <v>0.93</v>
       </c>
-      <c r="V24" s="41"/>
+      <c r="V24" s="39"/>
       <c r="W24" s="9" t="s">
         <v>30</v>
       </c>
@@ -5954,14 +5932,14 @@
         <v/>
       </c>
       <c r="AA24" s="20" t="str">
-        <f>IF(OR(S24="",Z24=""),"",S24-Z24)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB24" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.5">
+    <row r="25" spans="1:28" ht="26.4">
       <c r="A25" s="6" t="s">
         <v>78</v>
       </c>
@@ -5981,7 +5959,7 @@
         <v>40</v>
       </c>
       <c r="G25" s="18">
-        <f t="shared" ref="G25" si="7">ROUND(F25/0.8,0)</f>
+        <f t="shared" ref="G25" si="8">ROUND(F25/0.8,0)</f>
         <v>50</v>
       </c>
       <c r="H25" s="8" t="s">
@@ -6006,7 +5984,7 @@
         <v>2</v>
       </c>
       <c r="O25" s="20">
-        <f t="shared" ref="O25:O38" si="8">72*N25</f>
+        <f t="shared" ref="O25:O38" si="9">72*N25</f>
         <v>144</v>
       </c>
       <c r="P25" s="25" t="s">
@@ -6016,38 +5994,38 @@
         <v>0</v>
       </c>
       <c r="R25" s="24">
-        <f t="shared" ref="R25:R33" si="9">4*36*Q25</f>
+        <f t="shared" ref="R25:R33" si="10">4*36*Q25</f>
         <v>0</v>
       </c>
       <c r="S25" s="20">
-        <f t="shared" ref="S25:S38" si="10">O25</f>
+        <f t="shared" ref="S25:S38" si="11">O25</f>
         <v>144</v>
       </c>
       <c r="T25" s="29">
         <v>168</v>
       </c>
-      <c r="U25" s="42">
+      <c r="U25" s="40">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="V25" s="41"/>
+      <c r="V25" s="39"/>
       <c r="W25" s="9" t="s">
         <v>30</v>
       </c>
       <c r="X25" s="9"/>
       <c r="Y25" s="20"/>
       <c r="Z25" s="20" t="str">
-        <f t="shared" ref="Z25" si="11">IF(OR(X25="",Y25=""),"",X25*Y25)</f>
+        <f t="shared" ref="Z25" si="12">IF(OR(X25="",Y25=""),"",X25*Y25)</f>
         <v/>
       </c>
       <c r="AA25" s="20" t="str">
-        <f>IF(OR(S25="",Z25=""),"",S25-Z25)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB25" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.5">
+    <row r="26" spans="1:28" ht="26.4">
       <c r="A26" s="6" t="s">
         <v>78</v>
       </c>
@@ -6067,7 +6045,7 @@
         <v>80</v>
       </c>
       <c r="G26" s="18">
-        <f t="shared" ref="G26:G38" si="12">ROUND(F26/0.8,0)</f>
+        <f t="shared" ref="G26:G38" si="13">ROUND(F26/0.8,0)</f>
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
@@ -6092,7 +6070,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="P26" s="25" t="s">
@@ -6102,38 +6080,38 @@
         <v>0</v>
       </c>
       <c r="R26" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S26" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="T26" s="29">
         <v>0</v>
       </c>
-      <c r="U26" s="40">
-        <v>0</v>
-      </c>
-      <c r="V26" s="39"/>
+      <c r="U26" s="38">
+        <v>0</v>
+      </c>
+      <c r="V26" s="37"/>
       <c r="W26" s="9" t="s">
         <v>30</v>
       </c>
       <c r="X26" s="9"/>
       <c r="Y26" s="20"/>
       <c r="Z26" s="20" t="str">
-        <f t="shared" ref="Z26:Z38" si="13">IF(OR(X26="",Y26=""),"",X26*Y26)</f>
+        <f t="shared" ref="Z26:Z38" si="14">IF(OR(X26="",Y26=""),"",X26*Y26)</f>
         <v/>
       </c>
       <c r="AA26" s="20" t="str">
-        <f>IF(OR(S26="",Z26=""),"",S26-Z26)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB26" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="25.5">
+    <row r="27" spans="1:28" ht="26.4">
       <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
@@ -6153,7 +6131,7 @@
         <v>320</v>
       </c>
       <c r="G27" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H27" s="8" t="s">
@@ -6188,20 +6166,20 @@
         <v>0</v>
       </c>
       <c r="R27" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S27" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>288</v>
       </c>
       <c r="T27" s="29">
         <v>291</v>
       </c>
-      <c r="U27" s="42">
+      <c r="U27" s="40">
         <v>0.67</v>
       </c>
-      <c r="V27" s="43">
+      <c r="V27" s="41">
         <v>22</v>
       </c>
       <c r="W27" s="9" t="s">
@@ -6210,18 +6188,18 @@
       <c r="X27" s="9"/>
       <c r="Y27" s="20"/>
       <c r="Z27" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA27" s="20" t="str">
-        <f>IF(OR(S27="",Z27=""),"",S27-Z27)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB27" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.5">
+    <row r="28" spans="1:28" ht="26.4">
       <c r="A28" s="6" t="s">
         <v>78</v>
       </c>
@@ -6241,7 +6219,7 @@
         <v>320</v>
       </c>
       <c r="G28" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H28" s="8" t="s">
@@ -6266,7 +6244,7 @@
         <v>4</v>
       </c>
       <c r="O28" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>288</v>
       </c>
       <c r="P28" s="25" t="s">
@@ -6276,20 +6254,20 @@
         <v>0</v>
       </c>
       <c r="R28" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S28" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>288</v>
       </c>
       <c r="T28" s="29">
         <v>384</v>
       </c>
-      <c r="U28" s="38">
+      <c r="U28" s="36">
         <v>0.77</v>
       </c>
-      <c r="V28" s="43">
+      <c r="V28" s="41">
         <v>20.8</v>
       </c>
       <c r="W28" s="9" t="s">
@@ -6298,18 +6276,18 @@
       <c r="X28" s="9"/>
       <c r="Y28" s="20"/>
       <c r="Z28" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA28" s="20" t="str">
-        <f>IF(OR(S28="",Z28=""),"",S28-Z28)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="25.5">
+    <row r="29" spans="1:28" ht="26.4">
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
@@ -6329,7 +6307,7 @@
         <v>320</v>
       </c>
       <c r="G29" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H29" s="8" t="s">
@@ -6354,7 +6332,7 @@
         <v>5</v>
       </c>
       <c r="O29" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>360</v>
       </c>
       <c r="P29" s="25" t="s">
@@ -6364,20 +6342,20 @@
         <v>0</v>
       </c>
       <c r="R29" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S29" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>360</v>
       </c>
       <c r="T29" s="29">
         <v>375</v>
       </c>
-      <c r="U29" s="42">
+      <c r="U29" s="40">
         <v>0.59</v>
       </c>
-      <c r="V29" s="43">
+      <c r="V29" s="41">
         <v>22.6</v>
       </c>
       <c r="W29" s="9" t="s">
@@ -6386,18 +6364,18 @@
       <c r="X29" s="9"/>
       <c r="Y29" s="20"/>
       <c r="Z29" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA29" s="20" t="str">
-        <f>IF(OR(S29="",Z29=""),"",S29-Z29)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB29" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="25.5">
+    <row r="30" spans="1:28" ht="26.4">
       <c r="A30" s="6" t="s">
         <v>78</v>
       </c>
@@ -6417,7 +6395,7 @@
         <v>160</v>
       </c>
       <c r="G30" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>200</v>
       </c>
       <c r="H30" s="8" t="s">
@@ -6442,7 +6420,7 @@
         <v>7</v>
       </c>
       <c r="O30" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>504</v>
       </c>
       <c r="P30" s="25" t="s">
@@ -6452,20 +6430,20 @@
         <v>0</v>
       </c>
       <c r="R30" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S30" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>504</v>
       </c>
       <c r="T30" s="29">
         <v>316</v>
       </c>
-      <c r="U30" s="38">
+      <c r="U30" s="36">
         <v>0.62</v>
       </c>
-      <c r="V30" s="43">
+      <c r="V30" s="41">
         <v>25.1</v>
       </c>
       <c r="W30" s="9" t="s">
@@ -6474,18 +6452,18 @@
       <c r="X30" s="9"/>
       <c r="Y30" s="20"/>
       <c r="Z30" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA30" s="20" t="str">
-        <f>IF(OR(S30="",Z30=""),"",S30-Z30)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB30" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="25.5">
+    <row r="31" spans="1:28" ht="26.4">
       <c r="A31" s="6" t="s">
         <v>78</v>
       </c>
@@ -6505,7 +6483,7 @@
         <v>320</v>
       </c>
       <c r="G31" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H31" s="8" t="s">
@@ -6530,7 +6508,7 @@
         <v>9</v>
       </c>
       <c r="O31" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>648</v>
       </c>
       <c r="P31" s="25" t="s">
@@ -6540,20 +6518,20 @@
         <v>0</v>
       </c>
       <c r="R31" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S31" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>648</v>
       </c>
       <c r="T31" s="29">
         <v>476</v>
       </c>
-      <c r="U31" s="42">
+      <c r="U31" s="40">
         <v>0.66</v>
       </c>
-      <c r="V31" s="43">
+      <c r="V31" s="41">
         <v>21.4</v>
       </c>
       <c r="W31" s="9" t="s">
@@ -6562,18 +6540,18 @@
       <c r="X31" s="9"/>
       <c r="Y31" s="20"/>
       <c r="Z31" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA31" s="20" t="str">
-        <f>IF(OR(S31="",Z31=""),"",S31-Z31)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB31" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="25.5">
+    <row r="32" spans="1:28" ht="26.4">
       <c r="A32" s="6" t="s">
         <v>78</v>
       </c>
@@ -6593,7 +6571,7 @@
         <v>320</v>
       </c>
       <c r="G32" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H32" s="8" t="s">
@@ -6618,7 +6596,7 @@
         <v>6</v>
       </c>
       <c r="O32" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>432</v>
       </c>
       <c r="P32" s="25" t="s">
@@ -6628,20 +6606,20 @@
         <v>0</v>
       </c>
       <c r="R32" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S32" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>432</v>
       </c>
       <c r="T32" s="29">
         <v>552</v>
       </c>
-      <c r="U32" s="38">
+      <c r="U32" s="36">
         <v>0.72</v>
       </c>
-      <c r="V32" s="37">
+      <c r="V32" s="35">
         <v>18.5</v>
       </c>
       <c r="W32" s="9" t="s">
@@ -6650,18 +6628,18 @@
       <c r="X32" s="9"/>
       <c r="Y32" s="20"/>
       <c r="Z32" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA32" s="20" t="str">
-        <f>IF(OR(S32="",Z32=""),"",S32-Z32)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB32" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="25.5">
+    <row r="33" spans="1:28" ht="26.4">
       <c r="A33" s="6" t="s">
         <v>78</v>
       </c>
@@ -6681,7 +6659,7 @@
         <v>80</v>
       </c>
       <c r="G33" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
@@ -6706,7 +6684,7 @@
         <v>2</v>
       </c>
       <c r="O33" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>144</v>
       </c>
       <c r="P33" s="25" t="s">
@@ -6716,20 +6694,20 @@
         <v>0</v>
       </c>
       <c r="R33" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S33" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>144</v>
       </c>
       <c r="T33" s="29">
         <v>227</v>
       </c>
-      <c r="U33" s="38">
+      <c r="U33" s="36">
         <v>0.87</v>
       </c>
-      <c r="V33" s="37">
+      <c r="V33" s="35">
         <v>17.5</v>
       </c>
       <c r="W33" s="9" t="s">
@@ -6738,18 +6716,18 @@
       <c r="X33" s="9"/>
       <c r="Y33" s="20"/>
       <c r="Z33" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA33" s="20" t="str">
-        <f>IF(OR(S33="",Z33=""),"",S33-Z33)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB33" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="25.5">
+    <row r="34" spans="1:28" ht="26.4">
       <c r="A34" s="6" t="s">
         <v>78</v>
       </c>
@@ -6769,7 +6747,7 @@
         <v>320</v>
       </c>
       <c r="G34" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H34" s="8" t="s">
@@ -6794,7 +6772,7 @@
         <v>9</v>
       </c>
       <c r="O34" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>648</v>
       </c>
       <c r="P34" s="25" t="s">
@@ -6808,16 +6786,16 @@
         <v>0</v>
       </c>
       <c r="S34" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>648</v>
       </c>
       <c r="T34" s="29">
         <v>676</v>
       </c>
-      <c r="U34" s="42">
+      <c r="U34" s="40">
         <v>0.68</v>
       </c>
-      <c r="V34" s="43">
+      <c r="V34" s="41">
         <v>21.5</v>
       </c>
       <c r="W34" s="9" t="s">
@@ -6826,18 +6804,18 @@
       <c r="X34" s="9"/>
       <c r="Y34" s="20"/>
       <c r="Z34" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA34" s="20" t="str">
-        <f>IF(OR(S34="",Z34=""),"",S34-Z34)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB34" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="25.5">
+    <row r="35" spans="1:28" ht="26.4">
       <c r="A35" s="6" t="s">
         <v>78</v>
       </c>
@@ -6857,7 +6835,7 @@
         <v>80</v>
       </c>
       <c r="G35" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
@@ -6892,7 +6870,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="24">
-        <f t="shared" ref="R35:R38" si="14">4*36*Q35</f>
+        <f t="shared" ref="R35:R38" si="15">4*36*Q35</f>
         <v>0</v>
       </c>
       <c r="S35" s="20">
@@ -6902,10 +6880,10 @@
       <c r="T35" s="29">
         <v>273</v>
       </c>
-      <c r="U35" s="38">
+      <c r="U35" s="36">
         <v>0.66</v>
       </c>
-      <c r="V35" s="37">
+      <c r="V35" s="35">
         <v>21.1</v>
       </c>
       <c r="W35" s="9" t="s">
@@ -6914,18 +6892,18 @@
       <c r="X35" s="9"/>
       <c r="Y35" s="20"/>
       <c r="Z35" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA35" s="20" t="str">
-        <f>IF(OR(S35="",Z35=""),"",S35-Z35)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB35" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="25.5">
+    <row r="36" spans="1:28" ht="26.4">
       <c r="A36" s="6" t="s">
         <v>78</v>
       </c>
@@ -6945,7 +6923,7 @@
         <v>320</v>
       </c>
       <c r="G36" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H36" s="8" t="s">
@@ -6970,7 +6948,7 @@
         <v>8</v>
       </c>
       <c r="O36" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>576</v>
       </c>
       <c r="P36" s="25" t="s">
@@ -6980,20 +6958,20 @@
         <v>0</v>
       </c>
       <c r="R36" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="S36" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>576</v>
       </c>
       <c r="T36" s="29">
         <v>622</v>
       </c>
-      <c r="U36" s="38">
+      <c r="U36" s="36">
         <v>0.7</v>
       </c>
-      <c r="V36" s="37">
+      <c r="V36" s="35">
         <v>18.7</v>
       </c>
       <c r="W36" s="9" t="s">
@@ -7002,18 +6980,18 @@
       <c r="X36" s="9"/>
       <c r="Y36" s="20"/>
       <c r="Z36" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA36" s="20" t="str">
-        <f>IF(OR(S36="",Z36=""),"",S36-Z36)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB36" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="25.5">
+    <row r="37" spans="1:28" ht="26.4">
       <c r="A37" s="6" t="s">
         <v>78</v>
       </c>
@@ -7033,7 +7011,7 @@
         <v>80</v>
       </c>
       <c r="G37" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
@@ -7058,7 +7036,7 @@
         <v>1</v>
       </c>
       <c r="O37" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>72</v>
       </c>
       <c r="P37" s="25" t="s">
@@ -7068,20 +7046,20 @@
         <v>0</v>
       </c>
       <c r="R37" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="S37" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>72</v>
       </c>
       <c r="T37" s="29">
         <v>136</v>
       </c>
-      <c r="U37" s="38">
+      <c r="U37" s="36">
         <v>0.76</v>
       </c>
-      <c r="V37" s="37">
+      <c r="V37" s="35">
         <v>11.9</v>
       </c>
       <c r="W37" s="9" t="s">
@@ -7090,18 +7068,18 @@
       <c r="X37" s="9"/>
       <c r="Y37" s="20"/>
       <c r="Z37" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA37" s="20" t="str">
-        <f>IF(OR(S37="",Z37=""),"",S37-Z37)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB37" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:28" ht="25.5">
+    <row r="38" spans="1:28" ht="26.4">
       <c r="A38" s="11" t="s">
         <v>78</v>
       </c>
@@ -7121,7 +7099,7 @@
         <v>320</v>
       </c>
       <c r="G38" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H38" s="13" t="s">
@@ -7146,7 +7124,7 @@
         <v>8</v>
       </c>
       <c r="O38" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>576</v>
       </c>
       <c r="P38" s="25" t="s">
@@ -7156,20 +7134,20 @@
         <v>0</v>
       </c>
       <c r="R38" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="S38" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>576</v>
       </c>
       <c r="T38" s="29">
         <v>458</v>
       </c>
-      <c r="U38" s="42">
+      <c r="U38" s="40">
         <v>0.62</v>
       </c>
-      <c r="V38" s="43">
+      <c r="V38" s="41">
         <v>20.8</v>
       </c>
       <c r="W38" s="14" t="s">
@@ -7178,11 +7156,11 @@
       <c r="X38" s="14"/>
       <c r="Y38" s="21"/>
       <c r="Z38" s="21" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA38" s="21" t="str">
-        <f>IF(OR(S38="",Z38=""),"",S38-Z38)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB38" s="15" t="s">
@@ -7204,20 +7182,20 @@
     <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="T25">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$T25&gt;=$F25</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$T25&lt;$F25</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="T4:V23">
-    <cfRule type="expression" dxfId="7" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="4">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>$T4&lt;$F4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T25">
-    <cfRule type="expression" dxfId="5" priority="1">
-      <formula>$T25&gt;=$F25</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
-      <formula>$T25&lt;$F25</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7228,7 +7206,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
@@ -7236,19 +7214,19 @@
     <col min="6" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20.65">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:8" ht="21">
+      <c r="A1" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-    </row>
-    <row r="2" spans="1:8" ht="27.75">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+    </row>
+    <row r="2" spans="1:8" ht="27.6">
       <c r="A2" s="1" t="s">
         <v>148</v>
       </c>
@@ -7274,7 +7252,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="27">
+    <row r="3" spans="1:8" ht="27.6">
       <c r="A3" s="2" t="s">
         <v>69</v>
       </c>
@@ -7301,7 +7279,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="27">
+    <row r="4" spans="1:8" ht="27.6">
       <c r="A4" s="2" t="s">
         <v>158</v>
       </c>
@@ -7463,7 +7441,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="27">
+    <row r="10" spans="1:8" ht="27.6">
       <c r="A10" s="2" t="s">
         <v>174</v>
       </c>

</xml_diff>

<commit_message>
Addde univormity values for existing lighting in building A to excel
</commit_message>
<xml_diff>
--- a/Excel/Building_A_B_Carpark_Existing_Lighting.xlsx
+++ b/Excel/Building_A_B_Carpark_Existing_Lighting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liams\OneDrive\Documents\GitHub\Alpha_Design_17\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21969F3-485C-4FEC-9213-7728B3842F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314823BA-2A2C-4A27-8E53-AB6236D999CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="215">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -675,6 +675,9 @@
   </si>
   <si>
     <t>ACTUAL VALUES FOR BUILDING B GROUND FLOOR</t>
+  </si>
+  <si>
+    <t>Slope:0.41 Flat: 0.88</t>
   </si>
 </sst>
 </file>
@@ -965,7 +968,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1091,12 +1094,6 @@
     <xf numFmtId="164" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1116,6 +1113,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1351,36 +1358,37 @@
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="8.296875" customWidth="1"/>
     <col min="18" max="20" width="12" customWidth="1"/>
-    <col min="21" max="22" width="14" customWidth="1"/>
+    <col min="21" max="21" width="14" style="53" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="21">
-      <c r="A1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
+      <c r="A1" s="50" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
+      <c r="V1" s="50"/>
+      <c r="W1" s="50"/>
     </row>
     <row r="2" spans="1:28" ht="41.4">
       <c r="A2" s="3" t="s">
@@ -1525,7 +1533,9 @@
       <c r="T3" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="U3" s="27"/>
+      <c r="U3" s="27" t="s">
+        <v>214</v>
+      </c>
       <c r="V3" s="27"/>
       <c r="W3" s="9" t="s">
         <v>30</v>
@@ -1608,7 +1618,9 @@
       <c r="T4" s="27">
         <v>503</v>
       </c>
-      <c r="U4" s="27"/>
+      <c r="U4" s="52">
+        <v>0.46</v>
+      </c>
       <c r="V4" s="27"/>
       <c r="W4" s="9" t="s">
         <v>30</v>
@@ -1684,7 +1696,9 @@
       <c r="T5" s="27">
         <v>209</v>
       </c>
-      <c r="U5" s="27"/>
+      <c r="U5" s="52">
+        <v>0.9</v>
+      </c>
       <c r="V5" s="27"/>
       <c r="W5" s="9" t="s">
         <v>30</v>
@@ -1760,7 +1774,9 @@
       <c r="T6" s="27">
         <v>209</v>
       </c>
-      <c r="U6" s="27"/>
+      <c r="U6" s="52">
+        <v>0.89</v>
+      </c>
       <c r="V6" s="27"/>
       <c r="W6" s="9" t="s">
         <v>30</v>
@@ -1836,7 +1852,9 @@
       <c r="T7" s="27">
         <v>183</v>
       </c>
-      <c r="U7" s="27"/>
+      <c r="U7" s="52">
+        <v>0.84</v>
+      </c>
       <c r="V7" s="27"/>
       <c r="W7" s="9" t="s">
         <v>30</v>
@@ -1912,7 +1930,9 @@
       <c r="T8" s="27">
         <v>625</v>
       </c>
-      <c r="U8" s="27"/>
+      <c r="U8" s="52">
+        <v>0.57999999999999996</v>
+      </c>
       <c r="V8" s="27"/>
       <c r="W8" s="9" t="s">
         <v>56</v>
@@ -1988,7 +2008,9 @@
       <c r="T9" s="27">
         <v>644</v>
       </c>
-      <c r="U9" s="27"/>
+      <c r="U9" s="52">
+        <v>0.59</v>
+      </c>
       <c r="V9" s="27"/>
       <c r="W9" s="9" t="s">
         <v>56</v>
@@ -2071,7 +2093,9 @@
       <c r="T10" s="27">
         <v>373</v>
       </c>
-      <c r="U10" s="27"/>
+      <c r="U10" s="52">
+        <v>0.18</v>
+      </c>
       <c r="V10" s="27"/>
       <c r="W10" s="9" t="s">
         <v>30</v>
@@ -2147,7 +2171,9 @@
       <c r="T11" s="27">
         <v>615</v>
       </c>
-      <c r="U11" s="27"/>
+      <c r="U11" s="52">
+        <v>0.5</v>
+      </c>
       <c r="V11" s="27"/>
       <c r="W11" s="9" t="s">
         <v>56</v>
@@ -2222,7 +2248,9 @@
       <c r="T12" s="27">
         <v>836</v>
       </c>
-      <c r="U12" s="27"/>
+      <c r="U12" s="52">
+        <v>0.51</v>
+      </c>
       <c r="V12" s="27"/>
       <c r="W12" s="9" t="s">
         <v>56</v>
@@ -2298,7 +2326,9 @@
       <c r="T13" s="27">
         <v>743</v>
       </c>
-      <c r="U13" s="27"/>
+      <c r="U13" s="52">
+        <v>0.54</v>
+      </c>
       <c r="V13" s="42">
         <v>19.399999999999999</v>
       </c>
@@ -2376,7 +2406,9 @@
       <c r="T14" s="27">
         <v>1088</v>
       </c>
-      <c r="U14" s="27"/>
+      <c r="U14" s="52">
+        <v>0.5</v>
+      </c>
       <c r="V14" s="42">
         <v>19.5</v>
       </c>
@@ -2454,7 +2486,9 @@
       <c r="T15" s="27">
         <v>743</v>
       </c>
-      <c r="U15" s="27"/>
+      <c r="U15" s="52">
+        <v>0.41</v>
+      </c>
       <c r="V15" s="27"/>
       <c r="W15" s="9" t="s">
         <v>56</v>
@@ -2530,7 +2564,9 @@
       <c r="T16" s="27">
         <v>954</v>
       </c>
-      <c r="U16" s="27"/>
+      <c r="U16" s="52">
+        <v>0.5</v>
+      </c>
       <c r="V16" s="27"/>
       <c r="W16" s="9" t="s">
         <v>56</v>
@@ -2606,7 +2642,9 @@
       <c r="T17" s="27">
         <v>150</v>
       </c>
-      <c r="U17" s="27"/>
+      <c r="U17" s="52">
+        <v>0.89</v>
+      </c>
       <c r="V17" s="27"/>
       <c r="W17" s="9" t="s">
         <v>30</v>
@@ -2682,7 +2720,9 @@
       <c r="T18" s="27">
         <v>140</v>
       </c>
-      <c r="U18" s="27"/>
+      <c r="U18" s="52">
+        <v>0.46</v>
+      </c>
       <c r="V18" s="27"/>
       <c r="W18" s="9" t="s">
         <v>30</v>
@@ -2758,7 +2798,9 @@
       <c r="T19" s="27">
         <v>331</v>
       </c>
-      <c r="U19" s="27"/>
+      <c r="U19" s="52">
+        <v>0.85</v>
+      </c>
       <c r="V19" s="27"/>
       <c r="W19" s="9" t="s">
         <v>56</v>
@@ -2834,7 +2876,9 @@
       <c r="T20" s="27">
         <v>470</v>
       </c>
-      <c r="U20" s="27"/>
+      <c r="U20" s="52">
+        <v>0.53</v>
+      </c>
       <c r="V20" s="27"/>
       <c r="W20" s="9" t="s">
         <v>56</v>
@@ -2910,7 +2954,9 @@
       <c r="T21" s="27">
         <v>181</v>
       </c>
-      <c r="U21" s="27"/>
+      <c r="U21" s="52">
+        <v>0.35</v>
+      </c>
       <c r="V21" s="27"/>
       <c r="W21" s="9" t="s">
         <v>30</v>
@@ -2986,7 +3032,9 @@
       <c r="T22" s="27">
         <v>269</v>
       </c>
-      <c r="U22" s="27"/>
+      <c r="U22" s="52">
+        <v>0.92</v>
+      </c>
       <c r="V22" s="27"/>
       <c r="W22" s="9" t="s">
         <v>30</v>
@@ -3062,7 +3110,9 @@
       <c r="T23" s="27">
         <v>516</v>
       </c>
-      <c r="U23" s="27"/>
+      <c r="U23" s="52">
+        <v>0.61</v>
+      </c>
       <c r="V23" s="27"/>
       <c r="W23" s="9" t="s">
         <v>56</v>
@@ -3138,7 +3188,9 @@
       <c r="T24" s="27">
         <v>458</v>
       </c>
-      <c r="U24" s="27"/>
+      <c r="U24" s="52">
+        <v>0.82</v>
+      </c>
       <c r="V24" s="27"/>
       <c r="W24" s="9" t="s">
         <v>56</v>
@@ -3214,7 +3266,9 @@
       <c r="T25" s="27">
         <v>422</v>
       </c>
-      <c r="U25" s="27"/>
+      <c r="U25" s="52">
+        <v>0.81</v>
+      </c>
       <c r="V25" s="27"/>
       <c r="W25" s="9" t="s">
         <v>56</v>
@@ -3290,7 +3344,9 @@
       <c r="T26" s="27">
         <v>455</v>
       </c>
-      <c r="U26" s="27"/>
+      <c r="U26" s="52">
+        <v>0.68</v>
+      </c>
       <c r="V26" s="42">
         <v>22</v>
       </c>
@@ -3368,7 +3424,9 @@
       <c r="T27" s="27">
         <v>133</v>
       </c>
-      <c r="U27" s="27"/>
+      <c r="U27" s="52">
+        <v>0.4</v>
+      </c>
       <c r="V27" s="27"/>
       <c r="W27" s="9" t="s">
         <v>30</v>
@@ -3444,7 +3502,9 @@
       <c r="T28" s="27">
         <v>435</v>
       </c>
-      <c r="U28" s="27"/>
+      <c r="U28" s="52">
+        <v>0.66</v>
+      </c>
       <c r="V28" s="27"/>
       <c r="W28" s="9" t="s">
         <v>56</v>
@@ -3520,7 +3580,9 @@
       <c r="T29" s="27">
         <v>118</v>
       </c>
-      <c r="U29" s="27"/>
+      <c r="U29" s="52">
+        <v>0.18</v>
+      </c>
       <c r="V29" s="27"/>
       <c r="W29" s="9" t="s">
         <v>30</v>
@@ -3596,7 +3658,9 @@
       <c r="T30" s="27">
         <v>416</v>
       </c>
-      <c r="U30" s="27"/>
+      <c r="U30" s="52">
+        <v>0.73</v>
+      </c>
       <c r="V30" s="27"/>
       <c r="W30" s="9" t="s">
         <v>56</v>
@@ -3672,7 +3736,9 @@
       <c r="T31" s="27">
         <v>419</v>
       </c>
-      <c r="U31" s="27"/>
+      <c r="U31" s="52">
+        <v>0.73</v>
+      </c>
       <c r="V31" s="27"/>
       <c r="W31" s="9" t="s">
         <v>56</v>
@@ -3748,7 +3814,9 @@
       <c r="T32" s="27">
         <v>400</v>
       </c>
-      <c r="U32" s="27"/>
+      <c r="U32" s="52">
+        <v>0.71</v>
+      </c>
       <c r="V32" s="27"/>
       <c r="W32" s="9" t="s">
         <v>56</v>
@@ -3824,7 +3892,9 @@
       <c r="T33" s="27">
         <v>140</v>
       </c>
-      <c r="U33" s="27"/>
+      <c r="U33" s="52">
+        <v>0.91</v>
+      </c>
       <c r="V33" s="27"/>
       <c r="W33" s="9" t="s">
         <v>30</v>
@@ -3900,7 +3970,9 @@
       <c r="T34" s="27">
         <v>140</v>
       </c>
-      <c r="U34" s="27"/>
+      <c r="U34" s="52">
+        <v>0.72</v>
+      </c>
       <c r="V34" s="27"/>
       <c r="W34" s="9" t="s">
         <v>30</v>
@@ -3976,7 +4048,9 @@
       <c r="T35" s="27">
         <v>405</v>
       </c>
-      <c r="U35" s="27"/>
+      <c r="U35" s="52">
+        <v>0.8</v>
+      </c>
       <c r="V35" s="27"/>
       <c r="W35" s="9" t="s">
         <v>56</v>
@@ -4052,7 +4126,9 @@
       <c r="T36" s="27">
         <v>392</v>
       </c>
-      <c r="U36" s="27"/>
+      <c r="U36" s="52">
+        <v>0.77</v>
+      </c>
       <c r="V36" s="27"/>
       <c r="W36" s="14" t="s">
         <v>56</v>
@@ -4114,35 +4190,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="21.6" thickBot="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="50" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
-      <c r="Z1" s="43"/>
-      <c r="AD1" s="51" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
+      <c r="V1" s="50"/>
+      <c r="W1" s="50"/>
+      <c r="X1" s="50"/>
+      <c r="Y1" s="50"/>
+      <c r="Z1" s="50"/>
+      <c r="AD1" s="49" t="s">
         <v>213</v>
       </c>
     </row>
@@ -4231,46 +4307,46 @@
       <c r="AB2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="AD2" s="45" t="s">
+      <c r="AD2" s="43" t="s">
         <v>201</v>
       </c>
-      <c r="AE2" s="46" t="s">
+      <c r="AE2" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="AF2" s="46" t="s">
+      <c r="AF2" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="AG2" s="46" t="s">
+      <c r="AG2" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="AH2" s="46" t="s">
+      <c r="AH2" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="AI2" s="46" t="s">
+      <c r="AI2" s="44" t="s">
         <v>202</v>
       </c>
-      <c r="AJ2" s="46" t="s">
+      <c r="AJ2" s="44" t="s">
         <v>192</v>
       </c>
-      <c r="AK2" s="46" t="s">
+      <c r="AK2" s="44" t="s">
         <v>203</v>
       </c>
-      <c r="AL2" s="46" t="s">
+      <c r="AL2" s="44" t="s">
         <v>197</v>
       </c>
-      <c r="AM2" s="46" t="s">
+      <c r="AM2" s="44" t="s">
         <v>204</v>
       </c>
-      <c r="AN2" s="46" t="s">
+      <c r="AN2" s="44" t="s">
         <v>205</v>
       </c>
-      <c r="AO2" s="46" t="s">
+      <c r="AO2" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="AP2" s="46" t="s">
+      <c r="AP2" s="44" t="s">
         <v>207</v>
       </c>
-      <c r="AQ2" s="46" t="s">
+      <c r="AQ2" s="44" t="s">
         <v>208</v>
       </c>
     </row>
@@ -4357,42 +4433,42 @@
       <c r="AB3" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD3" s="47">
+      <c r="AD3" s="45">
         <v>101</v>
       </c>
-      <c r="AE3" s="48" t="s">
+      <c r="AE3" s="46" t="s">
         <v>209</v>
       </c>
-      <c r="AF3" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="49">
+      <c r="AF3" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="47">
         <v>80</v>
       </c>
-      <c r="AH3" s="49">
+      <c r="AH3" s="47">
         <v>100</v>
       </c>
-      <c r="AI3" s="49">
+      <c r="AI3" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ3" s="50"/>
-      <c r="AK3" s="48" t="s">
+      <c r="AJ3" s="48"/>
+      <c r="AK3" s="46" t="s">
         <v>210</v>
       </c>
-      <c r="AL3" s="48" t="s">
+      <c r="AL3" s="46" t="s">
         <v>211</v>
       </c>
-      <c r="AM3" s="50"/>
-      <c r="AN3" s="49">
+      <c r="AM3" s="48"/>
+      <c r="AN3" s="47">
         <v>1</v>
       </c>
-      <c r="AO3" s="49">
-        <v>0</v>
-      </c>
-      <c r="AP3" s="49">
+      <c r="AO3" s="47">
+        <v>0</v>
+      </c>
+      <c r="AP3" s="47">
         <v>76</v>
       </c>
-      <c r="AQ3" s="49">
+      <c r="AQ3" s="47">
         <v>62.7</v>
       </c>
     </row>
@@ -4479,42 +4555,42 @@
       <c r="AB4" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD4" s="47">
+      <c r="AD4" s="45">
         <v>102</v>
       </c>
-      <c r="AE4" s="48" t="s">
+      <c r="AE4" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="AF4" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="49">
+      <c r="AF4" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="47">
         <v>40</v>
       </c>
-      <c r="AH4" s="49">
+      <c r="AH4" s="47">
         <v>50</v>
       </c>
-      <c r="AI4" s="49">
+      <c r="AI4" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ4" s="50"/>
-      <c r="AK4" s="49">
+      <c r="AJ4" s="48"/>
+      <c r="AK4" s="47">
         <v>378</v>
       </c>
-      <c r="AL4" s="49">
+      <c r="AL4" s="47">
         <v>0.3</v>
       </c>
-      <c r="AM4" s="50"/>
-      <c r="AN4" s="49">
+      <c r="AM4" s="48"/>
+      <c r="AN4" s="47">
         <v>2</v>
       </c>
-      <c r="AO4" s="49">
+      <c r="AO4" s="47">
         <v>5</v>
       </c>
-      <c r="AP4" s="49">
+      <c r="AP4" s="47">
         <v>892</v>
       </c>
-      <c r="AQ4" s="49">
+      <c r="AQ4" s="47">
         <v>735.9</v>
       </c>
     </row>
@@ -4601,46 +4677,46 @@
       <c r="AB5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD5" s="47">
+      <c r="AD5" s="45">
         <v>103</v>
       </c>
-      <c r="AE5" s="48" t="s">
+      <c r="AE5" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="AF5" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="49">
+      <c r="AF5" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="47">
         <v>40</v>
       </c>
-      <c r="AH5" s="49">
+      <c r="AH5" s="47">
         <v>50</v>
       </c>
-      <c r="AI5" s="49">
+      <c r="AI5" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ5" s="49">
+      <c r="AJ5" s="47">
         <v>25</v>
       </c>
-      <c r="AK5" s="49">
+      <c r="AK5" s="47">
         <v>326</v>
       </c>
-      <c r="AL5" s="49">
+      <c r="AL5" s="47">
         <v>0.49</v>
       </c>
-      <c r="AM5" s="49">
+      <c r="AM5" s="47">
         <v>18</v>
       </c>
-      <c r="AN5" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="49">
+      <c r="AN5" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO5" s="47">
         <v>1</v>
       </c>
-      <c r="AP5" s="49">
+      <c r="AP5" s="47">
         <v>148</v>
       </c>
-      <c r="AQ5" s="49">
+      <c r="AQ5" s="47">
         <v>122.1</v>
       </c>
     </row>
@@ -4727,46 +4803,46 @@
       <c r="AB6" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD6" s="47">
+      <c r="AD6" s="45">
         <v>104</v>
       </c>
-      <c r="AE6" s="48" t="s">
+      <c r="AE6" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="AF6" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="49">
+      <c r="AF6" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="47">
         <v>8</v>
       </c>
-      <c r="AH6" s="49">
+      <c r="AH6" s="47">
         <v>100</v>
       </c>
-      <c r="AI6" s="49">
+      <c r="AI6" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ6" s="49">
+      <c r="AJ6" s="47">
         <v>25</v>
       </c>
-      <c r="AK6" s="49">
+      <c r="AK6" s="47">
         <v>200</v>
       </c>
-      <c r="AL6" s="49">
+      <c r="AL6" s="47">
         <v>0.81</v>
       </c>
-      <c r="AM6" s="49">
+      <c r="AM6" s="47">
         <v>15.4</v>
       </c>
-      <c r="AN6" s="49">
+      <c r="AN6" s="47">
         <v>1</v>
       </c>
-      <c r="AO6" s="49">
-        <v>0</v>
-      </c>
-      <c r="AP6" s="49">
+      <c r="AO6" s="47">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="47">
         <v>76</v>
       </c>
-      <c r="AQ6" s="49">
+      <c r="AQ6" s="47">
         <v>62.7</v>
       </c>
     </row>
@@ -4853,46 +4929,46 @@
       <c r="AB7" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD7" s="47">
+      <c r="AD7" s="45">
         <v>105</v>
       </c>
-      <c r="AE7" s="48" t="s">
+      <c r="AE7" s="46" t="s">
         <v>212</v>
       </c>
-      <c r="AF7" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="49">
+      <c r="AF7" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="47">
         <v>80</v>
       </c>
-      <c r="AH7" s="49">
+      <c r="AH7" s="47">
         <v>100</v>
       </c>
-      <c r="AI7" s="49">
+      <c r="AI7" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ7" s="49">
+      <c r="AJ7" s="47">
         <v>22</v>
       </c>
-      <c r="AK7" s="49">
+      <c r="AK7" s="47">
         <v>199</v>
       </c>
-      <c r="AL7" s="49">
+      <c r="AL7" s="47">
         <v>0.76</v>
       </c>
-      <c r="AM7" s="49">
+      <c r="AM7" s="47">
         <v>15.3</v>
       </c>
-      <c r="AN7" s="49">
+      <c r="AN7" s="47">
         <v>1</v>
       </c>
-      <c r="AO7" s="49">
-        <v>0</v>
-      </c>
-      <c r="AP7" s="49">
+      <c r="AO7" s="47">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="47">
         <v>76</v>
       </c>
-      <c r="AQ7" s="49">
+      <c r="AQ7" s="47">
         <v>62.7</v>
       </c>
     </row>
@@ -4979,46 +5055,46 @@
       <c r="AB8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD8" s="47">
+      <c r="AD8" s="45">
         <v>106</v>
       </c>
-      <c r="AE8" s="48" t="s">
+      <c r="AE8" s="46" t="s">
         <v>212</v>
       </c>
-      <c r="AF8" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG8" s="49">
+      <c r="AF8" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="47">
         <v>80</v>
       </c>
-      <c r="AH8" s="49">
+      <c r="AH8" s="47">
         <v>100</v>
       </c>
-      <c r="AI8" s="49">
+      <c r="AI8" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ8" s="49">
+      <c r="AJ8" s="47">
         <v>22</v>
       </c>
-      <c r="AK8" s="49">
+      <c r="AK8" s="47">
         <v>186</v>
       </c>
-      <c r="AL8" s="49">
+      <c r="AL8" s="47">
         <v>0.77</v>
       </c>
-      <c r="AM8" s="49">
+      <c r="AM8" s="47">
         <v>17.7</v>
       </c>
-      <c r="AN8" s="49">
+      <c r="AN8" s="47">
         <v>1</v>
       </c>
-      <c r="AO8" s="49">
-        <v>0</v>
-      </c>
-      <c r="AP8" s="49">
+      <c r="AO8" s="47">
+        <v>0</v>
+      </c>
+      <c r="AP8" s="47">
         <v>76</v>
       </c>
-      <c r="AQ8" s="49">
+      <c r="AQ8" s="47">
         <v>62.7</v>
       </c>
     </row>
@@ -5105,46 +5181,46 @@
       <c r="AB9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD9" s="47">
+      <c r="AD9" s="45">
         <v>107</v>
       </c>
-      <c r="AE9" s="48" t="s">
+      <c r="AE9" s="46" t="s">
         <v>116</v>
       </c>
-      <c r="AF9" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG9" s="49">
+      <c r="AF9" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="47">
         <v>160</v>
       </c>
-      <c r="AH9" s="49">
+      <c r="AH9" s="47">
         <v>200</v>
       </c>
-      <c r="AI9" s="49">
+      <c r="AI9" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ9" s="49">
+      <c r="AJ9" s="47">
         <v>22</v>
       </c>
-      <c r="AK9" s="49">
+      <c r="AK9" s="47">
         <v>185</v>
       </c>
-      <c r="AL9" s="49">
+      <c r="AL9" s="47">
         <v>0.72</v>
       </c>
-      <c r="AM9" s="49">
+      <c r="AM9" s="47">
         <v>18.5</v>
       </c>
-      <c r="AN9" s="49">
+      <c r="AN9" s="47">
         <v>1</v>
       </c>
-      <c r="AO9" s="49">
-        <v>0</v>
-      </c>
-      <c r="AP9" s="49">
+      <c r="AO9" s="47">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="47">
         <v>76</v>
       </c>
-      <c r="AQ9" s="49">
+      <c r="AQ9" s="47">
         <v>62.7</v>
       </c>
     </row>
@@ -5231,46 +5307,46 @@
       <c r="AB10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD10" s="47">
+      <c r="AD10" s="45">
         <v>108</v>
       </c>
-      <c r="AE10" s="48" t="s">
+      <c r="AE10" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="AF10" s="49">
+      <c r="AF10" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG10" s="49">
+      <c r="AG10" s="47">
         <v>320</v>
       </c>
-      <c r="AH10" s="49">
+      <c r="AH10" s="47">
         <v>400</v>
       </c>
-      <c r="AI10" s="49">
+      <c r="AI10" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ10" s="49">
+      <c r="AJ10" s="47">
         <v>19</v>
       </c>
-      <c r="AK10" s="49">
+      <c r="AK10" s="47">
         <v>759</v>
       </c>
-      <c r="AL10" s="49">
+      <c r="AL10" s="47">
         <v>0.39</v>
       </c>
-      <c r="AM10" s="49">
+      <c r="AM10" s="47">
         <v>20.3</v>
       </c>
-      <c r="AN10" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO10" s="49">
+      <c r="AN10" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO10" s="47">
         <v>4</v>
       </c>
-      <c r="AP10" s="49">
+      <c r="AP10" s="47">
         <v>592</v>
       </c>
-      <c r="AQ10" s="49">
+      <c r="AQ10" s="47">
         <v>488.4</v>
       </c>
     </row>
@@ -5357,46 +5433,46 @@
       <c r="AB11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD11" s="47">
+      <c r="AD11" s="45">
         <v>109</v>
       </c>
-      <c r="AE11" s="48" t="s">
+      <c r="AE11" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="AF11" s="49">
+      <c r="AF11" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG11" s="49">
+      <c r="AG11" s="47">
         <v>320</v>
       </c>
-      <c r="AH11" s="49">
+      <c r="AH11" s="47">
         <v>400</v>
       </c>
-      <c r="AI11" s="49">
+      <c r="AI11" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ11" s="49">
+      <c r="AJ11" s="47">
         <v>19</v>
       </c>
-      <c r="AK11" s="49">
+      <c r="AK11" s="47">
         <v>791</v>
       </c>
-      <c r="AL11" s="49">
+      <c r="AL11" s="47">
         <v>0.53</v>
       </c>
-      <c r="AM11" s="49">
+      <c r="AM11" s="47">
         <v>18.3</v>
       </c>
-      <c r="AN11" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO11" s="49">
+      <c r="AN11" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO11" s="47">
         <v>2</v>
       </c>
-      <c r="AP11" s="49">
+      <c r="AP11" s="47">
         <v>296</v>
       </c>
-      <c r="AQ11" s="49">
+      <c r="AQ11" s="47">
         <v>244.2</v>
       </c>
     </row>
@@ -5483,46 +5559,46 @@
       <c r="AB12" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD12" s="47">
+      <c r="AD12" s="45">
         <v>110</v>
       </c>
-      <c r="AE12" s="48" t="s">
+      <c r="AE12" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="AF12" s="49">
+      <c r="AF12" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG12" s="49">
+      <c r="AG12" s="47">
         <v>320</v>
       </c>
-      <c r="AH12" s="49">
+      <c r="AH12" s="47">
         <v>400</v>
       </c>
-      <c r="AI12" s="49">
+      <c r="AI12" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ12" s="49">
+      <c r="AJ12" s="47">
         <v>19</v>
       </c>
-      <c r="AK12" s="49">
+      <c r="AK12" s="47">
         <v>1109</v>
       </c>
-      <c r="AL12" s="49">
+      <c r="AL12" s="47">
         <v>0.34</v>
       </c>
-      <c r="AM12" s="49">
+      <c r="AM12" s="47">
         <v>20.2</v>
       </c>
-      <c r="AN12" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO12" s="49">
+      <c r="AN12" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO12" s="47">
         <v>6</v>
       </c>
-      <c r="AP12" s="49">
+      <c r="AP12" s="47">
         <v>888</v>
       </c>
-      <c r="AQ12" s="49">
+      <c r="AQ12" s="47">
         <v>732.6</v>
       </c>
     </row>
@@ -5609,46 +5685,46 @@
       <c r="AB13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD13" s="47">
+      <c r="AD13" s="45">
         <v>111</v>
       </c>
-      <c r="AE13" s="48" t="s">
+      <c r="AE13" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="AF13" s="49">
+      <c r="AF13" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG13" s="49">
+      <c r="AG13" s="47">
         <v>320</v>
       </c>
-      <c r="AH13" s="49">
+      <c r="AH13" s="47">
         <v>400</v>
       </c>
-      <c r="AI13" s="49">
+      <c r="AI13" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ13" s="49">
+      <c r="AJ13" s="47">
         <v>19</v>
       </c>
-      <c r="AK13" s="49">
+      <c r="AK13" s="47">
         <v>737</v>
       </c>
-      <c r="AL13" s="49">
+      <c r="AL13" s="47">
         <v>0.47</v>
       </c>
-      <c r="AM13" s="49">
+      <c r="AM13" s="47">
         <v>19.399999999999999</v>
       </c>
-      <c r="AN13" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO13" s="49">
+      <c r="AN13" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO13" s="47">
         <v>2</v>
       </c>
-      <c r="AP13" s="49">
+      <c r="AP13" s="47">
         <v>296</v>
       </c>
-      <c r="AQ13" s="49">
+      <c r="AQ13" s="47">
         <v>244.2</v>
       </c>
     </row>
@@ -5735,46 +5811,46 @@
       <c r="AB14" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD14" s="47">
+      <c r="AD14" s="45">
         <v>112</v>
       </c>
-      <c r="AE14" s="48" t="s">
+      <c r="AE14" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="AF14" s="49">
+      <c r="AF14" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG14" s="49">
+      <c r="AG14" s="47">
         <v>320</v>
       </c>
-      <c r="AH14" s="49">
+      <c r="AH14" s="47">
         <v>400</v>
       </c>
-      <c r="AI14" s="49">
+      <c r="AI14" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ14" s="49">
+      <c r="AJ14" s="47">
         <v>19</v>
       </c>
-      <c r="AK14" s="49">
+      <c r="AK14" s="47">
         <v>861</v>
       </c>
-      <c r="AL14" s="49">
+      <c r="AL14" s="47">
         <v>0.35</v>
       </c>
-      <c r="AM14" s="49">
+      <c r="AM14" s="47">
         <v>19.5</v>
       </c>
-      <c r="AN14" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO14" s="49">
+      <c r="AN14" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO14" s="47">
         <v>3</v>
       </c>
-      <c r="AP14" s="49">
+      <c r="AP14" s="47">
         <v>444</v>
       </c>
-      <c r="AQ14" s="49">
+      <c r="AQ14" s="47">
         <v>366.3</v>
       </c>
     </row>
@@ -5861,42 +5937,42 @@
       <c r="AB15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD15" s="47">
+      <c r="AD15" s="45">
         <v>113</v>
       </c>
-      <c r="AE15" s="48" t="s">
+      <c r="AE15" s="46" t="s">
         <v>118</v>
       </c>
-      <c r="AF15" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG15" s="49">
+      <c r="AF15" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG15" s="47">
         <v>40</v>
       </c>
-      <c r="AH15" s="49">
+      <c r="AH15" s="47">
         <v>50</v>
       </c>
-      <c r="AI15" s="49">
+      <c r="AI15" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ15" s="50"/>
-      <c r="AK15" s="49">
+      <c r="AJ15" s="48"/>
+      <c r="AK15" s="47">
         <v>405</v>
       </c>
-      <c r="AL15" s="49">
+      <c r="AL15" s="47">
         <v>0.57999999999999996</v>
       </c>
-      <c r="AM15" s="50"/>
-      <c r="AN15" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO15" s="49">
+      <c r="AM15" s="48"/>
+      <c r="AN15" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO15" s="47">
         <v>2</v>
       </c>
-      <c r="AP15" s="49">
+      <c r="AP15" s="47">
         <v>296</v>
       </c>
-      <c r="AQ15" s="49">
+      <c r="AQ15" s="47">
         <v>244.2</v>
       </c>
     </row>
@@ -5983,46 +6059,46 @@
       <c r="AB16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD16" s="47">
+      <c r="AD16" s="45">
         <v>114</v>
       </c>
-      <c r="AE16" s="48" t="s">
+      <c r="AE16" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="AF16" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="49">
+      <c r="AF16" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG16" s="47">
         <v>40</v>
       </c>
-      <c r="AH16" s="49">
+      <c r="AH16" s="47">
         <v>50</v>
       </c>
-      <c r="AI16" s="49">
+      <c r="AI16" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ16" s="49">
+      <c r="AJ16" s="47">
         <v>25</v>
       </c>
-      <c r="AK16" s="49">
+      <c r="AK16" s="47">
         <v>406</v>
       </c>
-      <c r="AL16" s="49">
+      <c r="AL16" s="47">
         <v>0.74</v>
       </c>
-      <c r="AM16" s="49">
+      <c r="AM16" s="47">
         <v>17.399999999999999</v>
       </c>
-      <c r="AN16" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO16" s="49">
+      <c r="AN16" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO16" s="47">
         <v>1</v>
       </c>
-      <c r="AP16" s="49">
+      <c r="AP16" s="47">
         <v>148</v>
       </c>
-      <c r="AQ16" s="49">
+      <c r="AQ16" s="47">
         <v>122.1</v>
       </c>
     </row>
@@ -6109,46 +6185,46 @@
       <c r="AB17" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD17" s="47">
+      <c r="AD17" s="45">
         <v>115</v>
       </c>
-      <c r="AE17" s="48" t="s">
+      <c r="AE17" s="46" t="s">
         <v>121</v>
       </c>
-      <c r="AF17" s="49">
+      <c r="AF17" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG17" s="49">
+      <c r="AG17" s="47">
         <v>320</v>
       </c>
-      <c r="AH17" s="49">
+      <c r="AH17" s="47">
         <v>400</v>
       </c>
-      <c r="AI17" s="49">
+      <c r="AI17" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ17" s="49">
+      <c r="AJ17" s="47">
         <v>19</v>
       </c>
-      <c r="AK17" s="49">
+      <c r="AK17" s="47">
         <v>1061</v>
       </c>
-      <c r="AL17" s="49">
+      <c r="AL17" s="47">
         <v>0.51</v>
       </c>
-      <c r="AM17" s="49">
+      <c r="AM17" s="47">
         <v>19.5</v>
       </c>
-      <c r="AN17" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO17" s="49">
+      <c r="AN17" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO17" s="47">
         <v>4</v>
       </c>
-      <c r="AP17" s="49">
+      <c r="AP17" s="47">
         <v>592</v>
       </c>
-      <c r="AQ17" s="49">
+      <c r="AQ17" s="47">
         <v>488.4</v>
       </c>
     </row>
@@ -6235,46 +6311,46 @@
       <c r="AB18" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD18" s="47">
+      <c r="AD18" s="45">
         <v>116</v>
       </c>
-      <c r="AE18" s="48" t="s">
+      <c r="AE18" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="AF18" s="49">
+      <c r="AF18" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG18" s="49">
+      <c r="AG18" s="47">
         <v>320</v>
       </c>
-      <c r="AH18" s="49">
+      <c r="AH18" s="47">
         <v>400</v>
       </c>
-      <c r="AI18" s="49">
+      <c r="AI18" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ18" s="49">
+      <c r="AJ18" s="47">
         <v>19</v>
       </c>
-      <c r="AK18" s="49">
+      <c r="AK18" s="47">
         <v>858</v>
       </c>
-      <c r="AL18" s="49">
+      <c r="AL18" s="47">
         <v>0.59</v>
       </c>
-      <c r="AM18" s="49">
+      <c r="AM18" s="47">
         <v>18.8</v>
       </c>
-      <c r="AN18" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO18" s="49">
+      <c r="AN18" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO18" s="47">
         <v>2</v>
       </c>
-      <c r="AP18" s="49">
+      <c r="AP18" s="47">
         <v>296</v>
       </c>
-      <c r="AQ18" s="49">
+      <c r="AQ18" s="47">
         <v>244.2</v>
       </c>
     </row>
@@ -6361,42 +6437,42 @@
       <c r="AB19" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD19" s="47">
+      <c r="AD19" s="45">
         <v>117</v>
       </c>
-      <c r="AE19" s="48" t="s">
+      <c r="AE19" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="AF19" s="49">
-        <v>0</v>
-      </c>
-      <c r="AG19" s="49">
+      <c r="AF19" s="47">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="47">
         <v>40</v>
       </c>
-      <c r="AH19" s="49">
+      <c r="AH19" s="47">
         <v>50</v>
       </c>
-      <c r="AI19" s="49">
+      <c r="AI19" s="47">
         <v>0.3</v>
       </c>
-      <c r="AJ19" s="50"/>
-      <c r="AK19" s="49">
+      <c r="AJ19" s="48"/>
+      <c r="AK19" s="47">
         <v>540</v>
       </c>
-      <c r="AL19" s="49">
+      <c r="AL19" s="47">
         <v>0.27</v>
       </c>
-      <c r="AM19" s="50"/>
-      <c r="AN19" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO19" s="49">
+      <c r="AM19" s="48"/>
+      <c r="AN19" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO19" s="47">
         <v>6</v>
       </c>
-      <c r="AP19" s="49">
+      <c r="AP19" s="47">
         <v>888</v>
       </c>
-      <c r="AQ19" s="49">
+      <c r="AQ19" s="47">
         <v>732.6</v>
       </c>
     </row>
@@ -6483,46 +6559,46 @@
       <c r="AB20" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD20" s="47">
+      <c r="AD20" s="45">
         <v>118</v>
       </c>
-      <c r="AE20" s="48" t="s">
+      <c r="AE20" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="AF20" s="49">
+      <c r="AF20" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG20" s="49">
+      <c r="AG20" s="47">
         <v>320</v>
       </c>
-      <c r="AH20" s="49">
+      <c r="AH20" s="47">
         <v>400</v>
       </c>
-      <c r="AI20" s="49">
+      <c r="AI20" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ20" s="49">
+      <c r="AJ20" s="47">
         <v>19</v>
       </c>
-      <c r="AK20" s="49">
+      <c r="AK20" s="47">
         <v>1060</v>
       </c>
-      <c r="AL20" s="49">
+      <c r="AL20" s="47">
         <v>0.56999999999999995</v>
       </c>
-      <c r="AM20" s="49">
+      <c r="AM20" s="47">
         <v>18.899999999999999</v>
       </c>
-      <c r="AN20" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO20" s="49">
+      <c r="AN20" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO20" s="47">
         <v>4</v>
       </c>
-      <c r="AP20" s="49">
+      <c r="AP20" s="47">
         <v>592</v>
       </c>
-      <c r="AQ20" s="49">
+      <c r="AQ20" s="47">
         <v>488.4</v>
       </c>
     </row>
@@ -6609,46 +6685,46 @@
       <c r="AB21" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD21" s="47">
+      <c r="AD21" s="45">
         <v>119</v>
       </c>
-      <c r="AE21" s="48" t="s">
+      <c r="AE21" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="AF21" s="49">
+      <c r="AF21" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG21" s="49">
+      <c r="AG21" s="47">
         <v>320</v>
       </c>
-      <c r="AH21" s="49">
+      <c r="AH21" s="47">
         <v>400</v>
       </c>
-      <c r="AI21" s="49">
+      <c r="AI21" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ21" s="49">
+      <c r="AJ21" s="47">
         <v>19</v>
       </c>
-      <c r="AK21" s="49">
+      <c r="AK21" s="47">
         <v>543</v>
       </c>
-      <c r="AL21" s="49">
+      <c r="AL21" s="47">
         <v>0.49</v>
       </c>
-      <c r="AM21" s="49">
+      <c r="AM21" s="47">
         <v>18.7</v>
       </c>
-      <c r="AN21" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO21" s="49">
+      <c r="AN21" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO21" s="47">
         <v>1</v>
       </c>
-      <c r="AP21" s="49">
+      <c r="AP21" s="47">
         <v>148</v>
       </c>
-      <c r="AQ21" s="49">
+      <c r="AQ21" s="47">
         <v>122.1</v>
       </c>
     </row>
@@ -6735,46 +6811,46 @@
       <c r="AB22" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD22" s="47">
+      <c r="AD22" s="45">
         <v>120</v>
       </c>
-      <c r="AE22" s="48" t="s">
+      <c r="AE22" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="AF22" s="49">
+      <c r="AF22" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG22" s="49">
+      <c r="AG22" s="47">
         <v>320</v>
       </c>
-      <c r="AH22" s="49">
+      <c r="AH22" s="47">
         <v>400</v>
       </c>
-      <c r="AI22" s="49">
+      <c r="AI22" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ22" s="49">
+      <c r="AJ22" s="47">
         <v>19</v>
       </c>
-      <c r="AK22" s="49">
+      <c r="AK22" s="47">
         <v>1127</v>
       </c>
-      <c r="AL22" s="49">
+      <c r="AL22" s="47">
         <v>0.54</v>
       </c>
-      <c r="AM22" s="49">
+      <c r="AM22" s="47">
         <v>19</v>
       </c>
-      <c r="AN22" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO22" s="49">
+      <c r="AN22" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO22" s="47">
         <v>4</v>
       </c>
-      <c r="AP22" s="49">
+      <c r="AP22" s="47">
         <v>592</v>
       </c>
-      <c r="AQ22" s="49">
+      <c r="AQ22" s="47">
         <v>488.4</v>
       </c>
     </row>
@@ -6861,46 +6937,46 @@
       <c r="AB23" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AD23" s="47">
+      <c r="AD23" s="45">
         <v>121</v>
       </c>
-      <c r="AE23" s="48" t="s">
+      <c r="AE23" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="AF23" s="49">
+      <c r="AF23" s="47">
         <v>0.7</v>
       </c>
-      <c r="AG23" s="49">
+      <c r="AG23" s="47">
         <v>320</v>
       </c>
-      <c r="AH23" s="49">
+      <c r="AH23" s="47">
         <v>400</v>
       </c>
-      <c r="AI23" s="49">
+      <c r="AI23" s="47">
         <v>0.7</v>
       </c>
-      <c r="AJ23" s="49">
+      <c r="AJ23" s="47">
         <v>19</v>
       </c>
-      <c r="AK23" s="49">
+      <c r="AK23" s="47">
         <v>900</v>
       </c>
-      <c r="AL23" s="49">
+      <c r="AL23" s="47">
         <v>0.53</v>
       </c>
-      <c r="AM23" s="49">
+      <c r="AM23" s="47">
         <v>19.2</v>
       </c>
-      <c r="AN23" s="49">
-        <v>0</v>
-      </c>
-      <c r="AO23" s="49">
+      <c r="AN23" s="47">
+        <v>0</v>
+      </c>
+      <c r="AO23" s="47">
         <v>2</v>
       </c>
-      <c r="AP23" s="49">
+      <c r="AP23" s="47">
         <v>296</v>
       </c>
-      <c r="AQ23" s="49">
+      <c r="AQ23" s="47">
         <v>244.2</v>
       </c>
     </row>
@@ -8266,16 +8342,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="51" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
     </row>
     <row r="2" spans="1:8" ht="27.6">
       <c r="A2" s="1" t="s">

</xml_diff>